<commit_message>
Skipped runners: at-pick DI margin + ADX columns; Fresh Buys sector fill
Omar 2026-07-29: the Top Skipped Runners block now shows what the buyer/
seller margin and raw ADX WERE on each recommendation day (Wilder-14 from
Yahoo daily bars, cached per pick in research/rec-day-dmi-cache.json so
nightly runs only compute new picks). Tooltips carry the winners-only
caveat. Fresh Buys Sector column now fills from the public-scanner call
that already feeds RSI/relvol/52wk - chart-read runs previously left it
blank.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-28.xlsx
+++ b/reports/universe_2026-07-28.xlsx
@@ -587,6 +587,18 @@
     <comment ref="T10" authorId="0" shapeId="0">
       <text>
         <t>Days since the pick.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="U10" authorId="0" shapeId="0">
+      <text>
+        <t>The buyer/seller margin (+DI - -DI) on the DAY this name was recommended - the state of the fight when the pick was made. Computed once from daily history and cached. Context only: measured 2026-07-28, the margin does not predict returns.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="V10" authorId="0" shapeId="0">
+      <text>
+        <t>Raw trend strength (ADX) on the recommendation day. The 7/29 look at the top-10 runners found birthdays of every kind - from 17 (below our own gate; PBF, the biggest runner) to 56. Winners-only sample: describes the pool, predicts nothing.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
@@ -1664,7 +1676,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28 19:19 local</t>
+          <t>2026-07-29 07:56 local</t>
         </is>
       </c>
     </row>
@@ -3183,6 +3195,16 @@
           <t>Days</t>
         </is>
       </c>
+      <c r="U10" s="29" t="inlineStr">
+        <is>
+          <t>Buyers vs Sellers @ Pick</t>
+        </is>
+      </c>
+      <c r="V10" s="29" t="inlineStr">
+        <is>
+          <t>ADX @ Pick</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="33" t="inlineStr">
@@ -3254,6 +3276,12 @@
       <c r="T11" s="47" t="n">
         <v>17</v>
       </c>
+      <c r="U11" s="49" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="V11" s="49" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="33" t="inlineStr">
@@ -3325,6 +3353,12 @@
       <c r="T12" s="47" t="n">
         <v>15</v>
       </c>
+      <c r="U12" s="49" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="V12" s="49" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="33" t="inlineStr">
@@ -3396,6 +3430,12 @@
       <c r="T13" s="47" t="n">
         <v>15</v>
       </c>
+      <c r="U13" s="49" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="V13" s="49" t="n">
+        <v>45.2</v>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="33" t="inlineStr">
@@ -3467,6 +3507,12 @@
       <c r="T14" s="47" t="n">
         <v>15</v>
       </c>
+      <c r="U14" s="49" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="V14" s="49" t="n">
+        <v>24.5</v>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="33" t="inlineStr">
@@ -3538,6 +3584,12 @@
       <c r="T15" s="47" t="n">
         <v>17</v>
       </c>
+      <c r="U15" s="49" t="n">
+        <v>20</v>
+      </c>
+      <c r="V15" s="49" t="n">
+        <v>21.1</v>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
@@ -3609,6 +3661,12 @@
       <c r="T16" s="47" t="n">
         <v>15</v>
       </c>
+      <c r="U16" s="49" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="V16" s="49" t="n">
+        <v>31.4</v>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="33" t="inlineStr">
@@ -3680,6 +3738,12 @@
       <c r="T17" s="47" t="n">
         <v>14</v>
       </c>
+      <c r="U17" s="49" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="V17" s="49" t="n">
+        <v>39.5</v>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="33" t="inlineStr">
@@ -3755,6 +3819,12 @@
       <c r="T18" s="47" t="n">
         <v>15</v>
       </c>
+      <c r="U18" s="49" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="V18" s="49" t="n">
+        <v>46.2</v>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="23" t="inlineStr">
@@ -3830,6 +3900,12 @@
       <c r="T19" s="47" t="n">
         <v>15</v>
       </c>
+      <c r="U19" s="49" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="V19" s="49" t="n">
+        <v>52.2</v>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="56" t="inlineStr">
@@ -3904,6 +3980,12 @@
       </c>
       <c r="T20" s="47" t="n">
         <v>12</v>
+      </c>
+      <c r="U20" s="49" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="V20" s="49" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -26497,7 +26579,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>2026-07-28 19:19 local</t>
+          <t>2026-07-29 07:56 local</t>
         </is>
       </c>
     </row>
@@ -28763,7 +28845,11 @@
       <c r="G2" s="20" t="n">
         <v>37.8</v>
       </c>
-      <c r="H2" s="19" t="n"/>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>Health Services</t>
+        </is>
+      </c>
       <c r="I2" s="19" t="inlineStr">
         <is>
           <t>2026-07-23</t>
@@ -28847,7 +28933,11 @@
       <c r="G3" s="20" t="n">
         <v>33.2</v>
       </c>
-      <c r="H3" s="19" t="n"/>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -28937,7 +29027,11 @@
       <c r="G4" s="20" t="n">
         <v>29.2</v>
       </c>
-      <c r="H4" s="19" t="n"/>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>Health Technology</t>
+        </is>
+      </c>
       <c r="I4" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -29027,7 +29121,11 @@
       <c r="G5" s="20" t="n">
         <v>35.8</v>
       </c>
-      <c r="H5" s="19" t="n"/>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>Consumer Non-Durables</t>
+        </is>
+      </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -29125,7 +29223,11 @@
       <c r="G6" s="20" t="n">
         <v>25.8</v>
       </c>
-      <c r="H6" s="19" t="n"/>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>Health Technology</t>
+        </is>
+      </c>
       <c r="I6" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -29215,7 +29317,11 @@
       <c r="G7" s="20" t="n">
         <v>25.3</v>
       </c>
-      <c r="H7" s="19" t="n"/>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Producer Manufacturing</t>
+        </is>
+      </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -29299,7 +29405,11 @@
       <c r="G8" s="20" t="n">
         <v>29.5</v>
       </c>
-      <c r="H8" s="19" t="n"/>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>Producer Manufacturing</t>
+        </is>
+      </c>
       <c r="I8" s="19" t="inlineStr">
         <is>
           <t>2026-07-21</t>
@@ -29389,7 +29499,11 @@
       <c r="G9" s="20" t="n">
         <v>35.2</v>
       </c>
-      <c r="H9" s="19" t="n"/>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Industrial Services</t>
+        </is>
+      </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -29479,7 +29593,11 @@
       <c r="G10" s="20" t="n">
         <v>21.4</v>
       </c>
-      <c r="H10" s="19" t="n"/>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
           <t>2026-07-22</t>
@@ -29563,7 +29681,11 @@
       <c r="G11" s="20" t="n">
         <v>21.4</v>
       </c>
-      <c r="H11" s="19" t="n"/>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Producer Manufacturing</t>
+        </is>
+      </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -29653,7 +29775,11 @@
       <c r="G12" s="20" t="n">
         <v>25.4</v>
       </c>
-      <c r="H12" s="19" t="n"/>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Health Technology</t>
+        </is>
+      </c>
       <c r="I12" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -29751,7 +29877,11 @@
       <c r="G13" s="20" t="n">
         <v>23.7</v>
       </c>
-      <c r="H13" s="19" t="n"/>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Commercial Services</t>
+        </is>
+      </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
           <t>2026-07-21</t>
@@ -29841,7 +29971,11 @@
       <c r="G14" s="20" t="n">
         <v>26.7</v>
       </c>
-      <c r="H14" s="19" t="n"/>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I14" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -29925,7 +30059,11 @@
       <c r="G15" s="20" t="n">
         <v>20.5</v>
       </c>
-      <c r="H15" s="19" t="n"/>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -30015,7 +30153,11 @@
       <c r="G16" s="20" t="n">
         <v>26.9</v>
       </c>
-      <c r="H16" s="19" t="n"/>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I16" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -30105,7 +30247,11 @@
       <c r="G17" s="20" t="n">
         <v>23.4</v>
       </c>
-      <c r="H17" s="19" t="n"/>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
       <c r="I17" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -30195,7 +30341,11 @@
       <c r="G18" s="20" t="n">
         <v>21.4</v>
       </c>
-      <c r="H18" s="19" t="n"/>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Consumer Non-Durables</t>
+        </is>
+      </c>
       <c r="I18" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -30279,7 +30429,11 @@
       <c r="G19" s="20" t="n">
         <v>22.4</v>
       </c>
-      <c r="H19" s="19" t="n"/>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -30377,7 +30531,11 @@
       <c r="G20" s="20" t="n">
         <v>21.2</v>
       </c>
-      <c r="H20" s="19" t="n"/>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I20" s="19" t="inlineStr">
         <is>
           <t>2026-07-23</t>
@@ -30469,7 +30627,11 @@
       <c r="G21" s="26" t="n">
         <v>24.4</v>
       </c>
-      <c r="H21" s="25" t="n"/>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Durables</t>
+        </is>
+      </c>
       <c r="I21" s="25" t="inlineStr">
         <is>
           <t>2026-07-22</t>
@@ -30559,7 +30721,11 @@
       <c r="G22" s="26" t="n">
         <v>29.2</v>
       </c>
-      <c r="H22" s="25" t="n"/>
+      <c r="H22" s="25" t="inlineStr">
+        <is>
+          <t>Commercial Services</t>
+        </is>
+      </c>
       <c r="I22" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -30657,7 +30823,11 @@
       <c r="G23" s="26" t="n">
         <v>28</v>
       </c>
-      <c r="H23" s="25" t="n"/>
+      <c r="H23" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I23" s="25" t="inlineStr">
         <is>
           <t>2026-07-23</t>
@@ -30741,7 +30911,11 @@
       <c r="G24" s="26" t="n">
         <v>34.9</v>
       </c>
-      <c r="H24" s="25" t="n"/>
+      <c r="H24" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I24" s="25" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -30825,7 +30999,11 @@
       <c r="G25" s="26" t="n">
         <v>19.5</v>
       </c>
-      <c r="H25" s="25" t="n"/>
+      <c r="H25" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Durables</t>
+        </is>
+      </c>
       <c r="I25" s="25" t="inlineStr">
         <is>
           <t>2026-07-21</t>
@@ -30917,7 +31095,11 @@
       <c r="G26" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="H26" s="25" t="n"/>
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
       <c r="I26" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -31001,7 +31183,11 @@
       <c r="G27" s="26" t="n">
         <v>19.2</v>
       </c>
-      <c r="H27" s="25" t="n"/>
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Durables</t>
+        </is>
+      </c>
       <c r="I27" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31091,7 +31277,11 @@
       <c r="G28" s="26" t="n">
         <v>20.7</v>
       </c>
-      <c r="H28" s="25" t="n"/>
+      <c r="H28" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I28" s="25" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -31175,7 +31365,11 @@
       <c r="G29" s="26" t="n">
         <v>40</v>
       </c>
-      <c r="H29" s="25" t="n"/>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I29" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31259,7 +31453,11 @@
       <c r="G30" s="26" t="n">
         <v>26.2</v>
       </c>
-      <c r="H30" s="25" t="n"/>
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I30" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31343,7 +31541,11 @@
       <c r="G31" s="26" t="n">
         <v>18.9</v>
       </c>
-      <c r="H31" s="25" t="n"/>
+      <c r="H31" s="25" t="inlineStr">
+        <is>
+          <t>Health Technology</t>
+        </is>
+      </c>
       <c r="I31" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31589,7 +31791,11 @@
       <c r="G34" s="26" t="n">
         <v>17.5</v>
       </c>
-      <c r="H34" s="25" t="n"/>
+      <c r="H34" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Non-Durables</t>
+        </is>
+      </c>
       <c r="I34" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31673,7 +31879,11 @@
       <c r="G35" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="H35" s="25" t="n"/>
+      <c r="H35" s="25" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
       <c r="I35" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31757,7 +31967,11 @@
       <c r="G36" s="26" t="n">
         <v>18.1</v>
       </c>
-      <c r="H36" s="25" t="n"/>
+      <c r="H36" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I36" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -31855,7 +32069,11 @@
       <c r="G37" s="26" t="n">
         <v>20.9</v>
       </c>
-      <c r="H37" s="25" t="n"/>
+      <c r="H37" s="25" t="inlineStr">
+        <is>
+          <t>Process Industries</t>
+        </is>
+      </c>
       <c r="I37" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -31939,7 +32157,11 @@
       <c r="G38" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="H38" s="25" t="n"/>
+      <c r="H38" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Durables</t>
+        </is>
+      </c>
       <c r="I38" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32031,7 +32253,11 @@
       <c r="G39" s="26" t="n">
         <v>27.7</v>
       </c>
-      <c r="H39" s="25" t="n"/>
+      <c r="H39" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I39" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32123,7 +32349,11 @@
       <c r="G40" s="26" t="n">
         <v>15.8</v>
       </c>
-      <c r="H40" s="25" t="n"/>
+      <c r="H40" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I40" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -32207,7 +32437,11 @@
       <c r="G41" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="H41" s="25" t="n"/>
+      <c r="H41" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I41" s="25" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -32297,7 +32531,11 @@
       <c r="G42" s="26" t="n">
         <v>22.9</v>
       </c>
-      <c r="H42" s="25" t="n"/>
+      <c r="H42" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I42" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32381,7 +32619,11 @@
       <c r="G43" s="26" t="n">
         <v>18.4</v>
       </c>
-      <c r="H43" s="25" t="n"/>
+      <c r="H43" s="25" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
       <c r="I43" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32465,7 +32707,11 @@
       <c r="G44" s="26" t="n">
         <v>18.2</v>
       </c>
-      <c r="H44" s="25" t="n"/>
+      <c r="H44" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I44" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32549,7 +32795,11 @@
       <c r="G45" s="26" t="n">
         <v>19.2</v>
       </c>
-      <c r="H45" s="25" t="n"/>
+      <c r="H45" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I45" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -32633,7 +32883,11 @@
       <c r="G46" s="26" t="n">
         <v>30.9</v>
       </c>
-      <c r="H46" s="25" t="n"/>
+      <c r="H46" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I46" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -32725,7 +32979,11 @@
       <c r="G47" s="26" t="n">
         <v>11.8</v>
       </c>
-      <c r="H47" s="25" t="n"/>
+      <c r="H47" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Non-Durables</t>
+        </is>
+      </c>
       <c r="I47" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32809,7 +33067,11 @@
       <c r="G48" s="26" t="n">
         <v>41.5</v>
       </c>
-      <c r="H48" s="25" t="n"/>
+      <c r="H48" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I48" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -32901,7 +33163,11 @@
       <c r="G49" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="H49" s="25" t="n"/>
+      <c r="H49" s="25" t="inlineStr">
+        <is>
+          <t>Non-Energy Minerals</t>
+        </is>
+      </c>
       <c r="I49" s="25" t="inlineStr">
         <is>
           <t>2026-07-22</t>
@@ -32991,7 +33257,11 @@
       <c r="G50" s="26" t="n">
         <v>13.9</v>
       </c>
-      <c r="H50" s="25" t="n"/>
+      <c r="H50" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I50" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33083,7 +33353,11 @@
       <c r="G51" s="26" t="n">
         <v>27.5</v>
       </c>
-      <c r="H51" s="25" t="n"/>
+      <c r="H51" s="25" t="inlineStr">
+        <is>
+          <t>Process Industries</t>
+        </is>
+      </c>
       <c r="I51" s="25" t="inlineStr">
         <is>
           <t>2026-07-23</t>
@@ -33173,7 +33447,11 @@
       <c r="G52" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="H52" s="25" t="n"/>
+      <c r="H52" s="25" t="inlineStr">
+        <is>
+          <t>Process Industries</t>
+        </is>
+      </c>
       <c r="I52" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33257,7 +33535,11 @@
       <c r="G53" s="26" t="n">
         <v>16.7</v>
       </c>
-      <c r="H53" s="25" t="n"/>
+      <c r="H53" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I53" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33349,7 +33631,11 @@
       <c r="G54" s="26" t="n">
         <v>16.6</v>
       </c>
-      <c r="H54" s="25" t="n"/>
+      <c r="H54" s="25" t="inlineStr">
+        <is>
+          <t>Health Technology</t>
+        </is>
+      </c>
       <c r="I54" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33433,7 +33719,11 @@
       <c r="G55" s="26" t="n">
         <v>21.8</v>
       </c>
-      <c r="H55" s="25" t="n"/>
+      <c r="H55" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I55" s="25" t="inlineStr">
         <is>
           <t>2026-07-21</t>
@@ -33517,7 +33807,11 @@
       <c r="G56" s="26" t="n">
         <v>15.6</v>
       </c>
-      <c r="H56" s="25" t="n"/>
+      <c r="H56" s="25" t="inlineStr">
+        <is>
+          <t>Distribution Services</t>
+        </is>
+      </c>
       <c r="I56" s="25" t="inlineStr">
         <is>
           <t>2026-07-21</t>
@@ -33607,7 +33901,11 @@
       <c r="G57" s="26" t="n">
         <v>32.3</v>
       </c>
-      <c r="H57" s="25" t="n"/>
+      <c r="H57" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I57" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33691,7 +33989,11 @@
       <c r="G58" s="26" t="n">
         <v>20.5</v>
       </c>
-      <c r="H58" s="25" t="n"/>
+      <c r="H58" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I58" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33853,7 +34155,11 @@
       <c r="G60" s="26" t="n">
         <v>17.9</v>
       </c>
-      <c r="H60" s="25" t="n"/>
+      <c r="H60" s="25" t="inlineStr">
+        <is>
+          <t>Technology Services</t>
+        </is>
+      </c>
       <c r="I60" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -33937,7 +34243,11 @@
       <c r="G61" s="26" t="n">
         <v>25.3</v>
       </c>
-      <c r="H61" s="25" t="n"/>
+      <c r="H61" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I61" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -34027,7 +34337,11 @@
       <c r="G62" s="26" t="n">
         <v>31.9</v>
       </c>
-      <c r="H62" s="25" t="n"/>
+      <c r="H62" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I62" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -34111,7 +34425,11 @@
       <c r="G63" s="26" t="n">
         <v>18.9</v>
       </c>
-      <c r="H63" s="25" t="n"/>
+      <c r="H63" s="25" t="inlineStr">
+        <is>
+          <t>Producer Manufacturing</t>
+        </is>
+      </c>
       <c r="I63" s="25" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -34201,7 +34519,11 @@
       <c r="G64" s="26" t="n">
         <v>19.9</v>
       </c>
-      <c r="H64" s="25" t="n"/>
+      <c r="H64" s="25" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I64" s="25" t="inlineStr">
         <is>
           <t>2026-07-23</t>
@@ -34285,7 +34607,11 @@
       <c r="G65" s="26" t="n">
         <v>18.7</v>
       </c>
-      <c r="H65" s="25" t="n"/>
+      <c r="H65" s="25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
       <c r="I65" s="25" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -34375,7 +34701,11 @@
       <c r="G66" s="26" t="n">
         <v>17.6</v>
       </c>
-      <c r="H66" s="25" t="n"/>
+      <c r="H66" s="25" t="inlineStr">
+        <is>
+          <t>Producer Manufacturing</t>
+        </is>
+      </c>
       <c r="I66" s="25" t="inlineStr">
         <is>
           <t>2026-07-22</t>
@@ -34465,7 +34795,11 @@
       <c r="G67" s="26" t="n">
         <v>13.3</v>
       </c>
-      <c r="H67" s="25" t="n"/>
+      <c r="H67" s="25" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
       <c r="I67" s="25" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -34555,7 +34889,11 @@
       <c r="G68" s="26" t="n">
         <v>19.9</v>
       </c>
-      <c r="H68" s="25" t="n"/>
+      <c r="H68" s="25" t="inlineStr">
+        <is>
+          <t>Producer Manufacturing</t>
+        </is>
+      </c>
       <c r="I68" s="25" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -34731,7 +35069,11 @@
       <c r="G70" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="H70" s="25" t="n"/>
+      <c r="H70" s="25" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I70" s="25" t="inlineStr">
         <is>
           <t>2026-07-22</t>
@@ -34971,7 +35313,11 @@
       <c r="G73" s="26" t="n">
         <v>26</v>
       </c>
-      <c r="H73" s="25" t="n"/>
+      <c r="H73" s="25" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
       <c r="I73" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -35055,7 +35401,11 @@
       <c r="G74" s="26" t="n">
         <v>23.1</v>
       </c>
-      <c r="H74" s="25" t="n"/>
+      <c r="H74" s="25" t="inlineStr">
+        <is>
+          <t>Electronic Technology</t>
+        </is>
+      </c>
       <c r="I74" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -35217,7 +35567,11 @@
       <c r="G76" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="H76" s="25" t="n"/>
+      <c r="H76" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I76" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -35301,7 +35655,11 @@
       <c r="G77" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="H77" s="25" t="n"/>
+      <c r="H77" s="25" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
       <c r="I77" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -35385,7 +35743,11 @@
       <c r="G78" s="26" t="n">
         <v>20.6</v>
       </c>
-      <c r="H78" s="25" t="n"/>
+      <c r="H78" s="25" t="inlineStr">
+        <is>
+          <t>Health Technology</t>
+        </is>
+      </c>
       <c r="I78" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -35547,7 +35909,11 @@
       <c r="G80" s="26" t="n">
         <v>17.8</v>
       </c>
-      <c r="H80" s="25" t="n"/>
+      <c r="H80" s="25" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
       <c r="I80" s="25" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -35631,7 +35997,11 @@
       <c r="G81" s="26" t="n">
         <v>15.7</v>
       </c>
-      <c r="H81" s="25" t="n"/>
+      <c r="H81" s="25" t="inlineStr">
+        <is>
+          <t>Non-Energy Minerals</t>
+        </is>
+      </c>
       <c r="I81" s="25" t="inlineStr">
         <is>
           <t>2026-07-22</t>

</xml_diff>